<commit_message>
.exe para consumidores de proyecto
</commit_message>
<xml_diff>
--- a/Template_HRC_Farmatodo.xlsx
+++ b/Template_HRC_Farmatodo.xlsx
@@ -469,9 +469,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="C2:I42"/>
+  <dimension ref="A1:I42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2" customWidth="1" min="1" max="1"/>
+    <col width="2" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="21" customWidth="1" min="8" max="8"/>
+    <col width="120" customWidth="1" min="9" max="9"/>
+  </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2">
       <c r="C2" t="inlineStr">
         <is>
@@ -487,6 +499,7 @@
         <v>10000061418</v>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="C4" s="4" t="inlineStr">
         <is>
@@ -494,6 +507,7 @@
         </is>
       </c>
     </row>
+    <row r="5"/>
     <row r="6">
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -544,6 +558,8 @@
         <v>0.5600000098347664</v>
       </c>
     </row>
+    <row r="9"/>
+    <row r="10"/>
     <row r="11">
       <c r="C11" s="2" t="inlineStr">
         <is>
@@ -571,7 +587,7 @@
         <v>10000061418</v>
       </c>
       <c r="D12" s="5" t="n">
-        <v>45904</v>
+        <v>45905</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -582,6 +598,11 @@
         <v>1</v>
       </c>
     </row>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
     <row r="18">
       <c r="C18" s="6" t="inlineStr">
         <is>

</xml_diff>